<commit_message>
Process.xaml Updated. Config.xlsx Updated.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\RPA\CompaniesHouse\Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDAD445F-D91D-4D37-A49E-E0C357D85BBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CAF740D-B03E-4423-B18F-1EBA98284581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34669" yWindow="-109" windowWidth="26300" windowHeight="14169" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34669" yWindow="-109" windowWidth="26300" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="57">
   <si>
     <t>Name</t>
   </si>
@@ -187,6 +187,15 @@
   </si>
   <si>
     <t>SearchLink</t>
+  </si>
+  <si>
+    <t>StorageBucketFolder</t>
+  </si>
+  <si>
+    <t>StorageBucketName</t>
+  </si>
+  <si>
+    <t>CompaniesHouse_Stanislav_Output</t>
   </si>
 </sst>
 </file>
@@ -648,44 +657,58 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.3" customHeight="1">
-      <c r="A6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" t="s">
-        <v>48</v>
-      </c>
-    </row>
+    <row r="6" spans="1:26" ht="14.3" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.3" customHeight="1">
       <c r="A7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7">
-        <v>0.3</v>
+        <v>55</v>
+      </c>
+      <c r="B7" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.3" customHeight="1">
       <c r="A8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8">
-        <v>0.5</v>
+        <v>54</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.3" customHeight="1">
       <c r="A9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.3" customHeight="1">
+      <c r="A10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.3" customHeight="1">
+      <c r="A11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.3" customHeight="1">
+      <c r="A12" t="s">
         <v>51</v>
       </c>
-      <c r="B9">
+      <c r="B12">
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.3" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.3" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.3" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.3" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.3" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.3" customHeight="1"/>
@@ -1676,9 +1699,10 @@
   <phoneticPr fontId="2"/>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{F76B710B-51F9-4404-BA9B-6A8552B0B447}"/>
+    <hyperlink ref="B8" r:id="rId2" xr:uid="{5E7C0C86-5337-42D1-A845-054D38BC770C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>